<commit_message>
Update on home page
Signed-off-by: leenaS-d <leenaraju7198@gmail.com>
</commit_message>
<xml_diff>
--- a/RDK8/RDK8-comonents-catalog.xlsx
+++ b/RDK8/RDK8-comonents-catalog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ldhana149\RDKE-components-registry\RDK8\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF63862B-671C-4031-9A16-0F973FB5C7BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADFB30E0-C815-4976-AE3D-511F0D3B47F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{25E4EBF0-253B-4C9C-998E-FB08C73FD49A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="231">
   <si>
     <t>COMPONENTS</t>
   </si>
@@ -299,6 +299,9 @@
     <t>https://github.com/rdkcentral/entservices-messagecontrol/releases/tag/1.0.3</t>
   </si>
   <si>
+    <t>2.0.2</t>
+  </si>
+  <si>
     <t>entservices-monitor</t>
   </si>
   <si>
@@ -437,6 +440,12 @@
     <t>https://github.com/rdkcentral/entservices-usersettings/releases/tag/1.0.6</t>
   </si>
   <si>
+    <t>entservices-xcast</t>
+  </si>
+  <si>
+    <t>https://github.com/rdkcentral/entservices-xcast/releases/tag/2.0.2</t>
+  </si>
+  <si>
     <t>hdmicec</t>
   </si>
   <si>
@@ -518,6 +527,9 @@
     <t>https://github.com/rdkcentral/libSyscallWrapper</t>
   </si>
   <si>
+    <t>3.4.2</t>
+  </si>
+  <si>
     <t>memcr</t>
   </si>
   <si>
@@ -714,6 +726,12 @@
   </si>
   <si>
     <t>https://www.bluez.org</t>
+  </si>
+  <si>
+    <t>entservices-apis</t>
+  </si>
+  <si>
+    <t>https://github.com/rdkcentral/entservices-apis/releases/tag/3.4.2</t>
   </si>
 </sst>
 </file>
@@ -863,7 +881,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -880,6 +898,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1268,7 +1289,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8248C6F-D34E-4152-91E6-D60E20A6E179}">
-  <dimension ref="A1:F79"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.26953125" customWidth="1"/>
@@ -1309,10 +1330,10 @@
       <c r="C2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F2" s="5" t="s">
@@ -1329,14 +1350,14 @@
       <c r="C3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F3" s="24" t="s">
-        <v>219</v>
+      <c r="E3" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="25" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="29" x14ac:dyDescent="0.35">
@@ -1349,30 +1370,30 @@
       <c r="C4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="F4" s="26" t="s">
-        <v>224</v>
+      <c r="E4" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="27" t="s">
+        <v>228</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="13" t="s">
         <v>15</v>
       </c>
       <c r="D5" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="14" t="s">
         <v>7</v>
       </c>
       <c r="F5" s="5" t="s">
@@ -1389,10 +1410,10 @@
       <c r="C6" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F6" s="5" t="s">
@@ -1403,16 +1424,16 @@
       <c r="A7" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="13" t="s">
         <v>29</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F7" s="5" t="s">
@@ -1420,17 +1441,17 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="15" t="s">
+      <c r="C8" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="16"/>
-      <c r="E8" s="17" t="s">
+      <c r="D8" s="17"/>
+      <c r="E8" s="18" t="s">
         <v>7</v>
       </c>
       <c r="F8" s="5" t="s">
@@ -1441,16 +1462,16 @@
       <c r="A9" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" s="8" t="s">
+      <c r="C9" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F9" s="5" t="s">
@@ -1461,10 +1482,10 @@
       <c r="A10" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="13" t="s">
         <v>6</v>
       </c>
       <c r="D10" s="1" t="s">
@@ -1481,16 +1502,16 @@
       <c r="A11" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="12" t="s">
+      <c r="C11" s="13" t="s">
         <v>6</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="E11" s="14" t="s">
         <v>7</v>
       </c>
       <c r="F11" s="5" t="s">
@@ -1501,16 +1522,16 @@
       <c r="A12" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="13" t="s">
         <v>43</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="E12" s="12" t="s">
         <v>7</v>
       </c>
       <c r="F12" s="5" t="s">
@@ -1521,16 +1542,16 @@
       <c r="A13" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="13" t="s">
         <v>43</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="E13" s="12" t="s">
         <v>7</v>
       </c>
       <c r="F13" s="5" t="s">
@@ -1541,16 +1562,16 @@
       <c r="A14" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="13" t="s">
         <v>43</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="E14" s="11" t="s">
+      <c r="E14" s="12" t="s">
         <v>7</v>
       </c>
       <c r="F14" s="5" t="s">
@@ -1561,16 +1582,16 @@
       <c r="A15" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="13" t="s">
         <v>43</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F15" s="5" t="s">
@@ -1581,16 +1602,16 @@
       <c r="A16" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="B16" s="13" t="s">
         <v>43</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="E16" s="9" t="s">
+      <c r="E16" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F16" s="5" t="s">
@@ -1601,16 +1622,16 @@
       <c r="A17" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="B17" s="13" t="s">
         <v>43</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="E17" s="11" t="s">
+      <c r="E17" s="12" t="s">
         <v>7</v>
       </c>
       <c r="F17" s="5" t="s">
@@ -1621,16 +1642,16 @@
       <c r="A18" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="13" t="s">
         <v>43</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="D18" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="E18" s="9" t="s">
+      <c r="E18" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F18" s="5" t="s">
@@ -1641,16 +1662,16 @@
       <c r="A19" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B19" s="12" t="s">
+      <c r="B19" s="13" t="s">
         <v>43</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="E19" s="11" t="s">
+      <c r="E19" s="12" t="s">
         <v>7</v>
       </c>
       <c r="F19" s="5" t="s">
@@ -1661,16 +1682,16 @@
       <c r="A20" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B20" s="12" t="s">
+      <c r="B20" s="13" t="s">
         <v>43</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D20" s="8" t="s">
+      <c r="D20" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="E20" s="9" t="s">
+      <c r="E20" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F20" s="5" t="s">
@@ -1681,16 +1702,16 @@
       <c r="A21" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="B21" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="C21" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="D21" s="8" t="s">
+      <c r="B21" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="D21" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="E21" s="9" t="s">
+      <c r="E21" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F21" s="5" t="s">
@@ -1701,16 +1722,16 @@
       <c r="A22" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="B22" s="12" t="s">
+      <c r="B22" s="13" t="s">
         <v>43</v>
       </c>
       <c r="C22" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D22" s="8" t="s">
+      <c r="D22" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="E22" s="9" t="s">
+      <c r="E22" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F22" s="5" t="s">
@@ -1721,16 +1742,16 @@
       <c r="A23" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B23" s="12" t="s">
+      <c r="B23" s="13" t="s">
         <v>43</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="D23" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="E23" s="11" t="s">
+      <c r="E23" s="12" t="s">
         <v>7</v>
       </c>
       <c r="F23" s="5" t="s">
@@ -1741,16 +1762,16 @@
       <c r="A24" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B24" s="12" t="s">
+      <c r="B24" s="13" t="s">
         <v>43</v>
       </c>
       <c r="C24" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="D24" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="E24" s="9" t="s">
+      <c r="E24" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F24" s="5" t="s">
@@ -1761,16 +1782,16 @@
       <c r="A25" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="B25" s="12" t="s">
+      <c r="B25" s="13" t="s">
         <v>43</v>
       </c>
       <c r="C25" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D25" s="8" t="s">
+      <c r="D25" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E25" s="9" t="s">
+      <c r="E25" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F25" s="5" t="s">
@@ -1781,16 +1802,16 @@
       <c r="A26" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B26" s="12" t="s">
+      <c r="B26" s="13" t="s">
         <v>43</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D26" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="E26" s="11" t="s">
+      <c r="E26" s="12" t="s">
         <v>7</v>
       </c>
       <c r="F26" s="5" t="s">
@@ -1799,169 +1820,169 @@
     </row>
     <row r="27" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A27" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="B27" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="B27" s="13" t="s">
         <v>43</v>
       </c>
       <c r="C27" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D27" s="8" t="s">
+      <c r="D27" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="E27" s="9" t="s">
+      <c r="E27" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="B28" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="B28" s="13" t="s">
         <v>43</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D28" s="10" t="s">
+      <c r="D28" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="E28" s="11" t="s">
+      <c r="E28" s="12" t="s">
         <v>7</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A29" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="B29" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="B29" s="13" t="s">
         <v>43</v>
       </c>
       <c r="C29" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D29" s="8" t="s">
+      <c r="D29" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="E29" s="9" t="s">
+      <c r="E29" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="B30" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="B30" s="13" t="s">
         <v>43</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D30" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="E30" s="11" t="s">
+      <c r="D30" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="E30" s="12" t="s">
         <v>7</v>
       </c>
       <c r="F30" s="5" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="58" x14ac:dyDescent="0.35">
+      <c r="A31" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="B31" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="D31" s="19" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" ht="58" x14ac:dyDescent="0.35">
-      <c r="A31" s="15" t="s">
+      <c r="E31" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="F31" s="5" t="s">
         <v>95</v>
-      </c>
-      <c r="B31" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="C31" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="D31" s="18" t="s">
-        <v>93</v>
-      </c>
-      <c r="E31" s="17" t="s">
-        <v>7</v>
-      </c>
-      <c r="F31" s="5" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="B32" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="B32" s="13" t="s">
         <v>43</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D32" s="10" t="s">
+      <c r="D32" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="E32" s="11" t="s">
+      <c r="E32" s="12" t="s">
         <v>7</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A33" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B33" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="B33" s="13" t="s">
         <v>43</v>
       </c>
       <c r="C33" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D33" s="8" t="s">
+      <c r="D33" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="E33" s="9" t="s">
+      <c r="E33" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="B34" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="B34" s="13" t="s">
         <v>43</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D34" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="E34" s="11" t="s">
+      <c r="D34" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="E34" s="12" t="s">
         <v>7</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A35" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="B35" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="B35" s="13" t="s">
         <v>43</v>
       </c>
       <c r="C35" s="6" t="s">
@@ -1970,36 +1991,36 @@
       <c r="D35" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E35" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="F35" s="14" t="s">
-        <v>104</v>
+      <c r="E35" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="F35" s="15" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="B36" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="B36" s="13" t="s">
         <v>43</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D36" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="E36" s="11" t="s">
+      <c r="D36" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="E36" s="12" t="s">
         <v>7</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A37" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B37" s="6" t="s">
         <v>43</v>
@@ -2007,19 +2028,19 @@
       <c r="C37" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D37" s="8" t="s">
+      <c r="D37" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="E37" s="9" t="s">
+      <c r="E37" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>43</v>
@@ -2027,19 +2048,19 @@
       <c r="C38" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D38" s="10" t="s">
+      <c r="D38" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="E38" s="11" t="s">
+      <c r="E38" s="12" t="s">
         <v>7</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A39" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B39" s="6" t="s">
         <v>43</v>
@@ -2047,19 +2068,19 @@
       <c r="C39" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D39" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="E39" s="9" t="s">
+      <c r="D39" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="E39" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>43</v>
@@ -2067,19 +2088,19 @@
       <c r="C40" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D40" s="10" t="s">
+      <c r="D40" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="E40" s="11" t="s">
+      <c r="E40" s="12" t="s">
         <v>7</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A41" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B41" s="6" t="s">
         <v>43</v>
@@ -2087,19 +2108,19 @@
       <c r="C41" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D41" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="E41" s="9" t="s">
+      <c r="D41" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="E41" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>43</v>
@@ -2107,19 +2128,19 @@
       <c r="C42" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D42" s="10" t="s">
+      <c r="D42" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="E42" s="11" t="s">
+      <c r="E42" s="12" t="s">
         <v>7</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A43" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B43" s="6" t="s">
         <v>43</v>
@@ -2127,19 +2148,19 @@
       <c r="C43" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D43" s="8" t="s">
+      <c r="D43" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="E43" s="9" t="s">
+      <c r="E43" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>43</v>
@@ -2147,19 +2168,19 @@
       <c r="C44" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D44" s="10" t="s">
+      <c r="D44" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="E44" s="11" t="s">
+      <c r="E44" s="12" t="s">
         <v>7</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A45" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B45" s="6" t="s">
         <v>43</v>
@@ -2167,19 +2188,19 @@
       <c r="C45" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D45" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="E45" s="9" t="s">
+      <c r="D45" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="E45" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>43</v>
@@ -2187,39 +2208,39 @@
       <c r="C46" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D46" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="E46" s="11" t="s">
+      <c r="D46" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="E46" s="12" t="s">
         <v>7</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A47" s="15" t="s">
-        <v>132</v>
-      </c>
-      <c r="B47" s="12" t="s">
+      <c r="A47" s="16" t="s">
+        <v>135</v>
+      </c>
+      <c r="B47" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C47" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="D47" s="18" t="s">
-        <v>133</v>
-      </c>
-      <c r="E47" s="17" t="s">
+      <c r="C47" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="D47" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="E47" s="18" t="s">
         <v>7</v>
       </c>
       <c r="F47" s="5" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A48" s="6" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B48" s="6" t="s">
         <v>31</v>
@@ -2227,39 +2248,39 @@
       <c r="C48" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D48" s="8" t="s">
+      <c r="D48" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="E48" s="9" t="s">
+      <c r="E48" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="B49" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="B49" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="C49" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="D49" s="10" t="s">
-        <v>138</v>
-      </c>
-      <c r="E49" s="11" t="s">
+      <c r="C49" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="D49" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="E49" s="12" t="s">
         <v>7</v>
       </c>
       <c r="F49" s="5" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>23</v>
@@ -2274,112 +2295,112 @@
         <v>7</v>
       </c>
       <c r="F50" s="5" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="6" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="C51" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="E51" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="F51" s="14" t="s">
-        <v>144</v>
+        <v>146</v>
+      </c>
+      <c r="E51" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="F51" s="15" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D52" s="10" t="s">
+      <c r="D52" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="E52" s="11" t="s">
+      <c r="E52" s="12" t="s">
         <v>7</v>
       </c>
       <c r="F52" s="5" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="B53" s="12" t="s">
-        <v>149</v>
+        <v>151</v>
+      </c>
+      <c r="B53" s="13" t="s">
+        <v>152</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>7</v>
       </c>
       <c r="F53" s="5" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="54" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A54" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="B54" s="19" t="s">
+        <v>155</v>
+      </c>
+      <c r="B54" s="20" t="s">
+        <v>156</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D54" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="C54" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="D54" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="E54" s="13" t="s">
+      <c r="E54" s="14" t="s">
         <v>7</v>
       </c>
       <c r="F54" s="5" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="55" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B55" s="12" t="s">
+        <v>157</v>
+      </c>
+      <c r="B55" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D55" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="E55" s="11" t="s">
+      <c r="D55" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="E55" s="12" t="s">
         <v>7</v>
       </c>
       <c r="F55" s="5" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
     </row>
     <row r="56" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A56" s="6" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B56" s="6" t="s">
         <v>23</v>
@@ -2388,20 +2409,20 @@
         <v>6</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="E56" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="E56" s="14" t="s">
         <v>7</v>
       </c>
       <c r="F56" s="5" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
     </row>
     <row r="57" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="B57" s="19" t="s">
+        <v>163</v>
+      </c>
+      <c r="B57" s="20" t="s">
         <v>42</v>
       </c>
       <c r="C57" s="1" t="s">
@@ -2413,33 +2434,33 @@
       <c r="E57" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F57" s="14" t="s">
-        <v>160</v>
+      <c r="F57" s="15" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="58" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="C58" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="C58" s="13" t="s">
         <v>6</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>7</v>
       </c>
       <c r="F58" s="5" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="59" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A59" s="6" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B59" s="6" t="s">
         <v>31</v>
@@ -2448,158 +2469,158 @@
         <v>6</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="E59" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="E59" s="14" t="s">
         <v>7</v>
       </c>
       <c r="F59" s="5" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
     </row>
     <row r="60" spans="1:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="A60" s="15" t="s">
-        <v>170</v>
-      </c>
-      <c r="B60" s="15" t="s">
+      <c r="A60" s="16" t="s">
+        <v>174</v>
+      </c>
+      <c r="B60" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="C60" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="D60" s="15" t="s">
-        <v>171</v>
-      </c>
-      <c r="E60" s="20" t="s">
+      <c r="C60" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="D60" s="16" t="s">
+        <v>175</v>
+      </c>
+      <c r="E60" s="21" t="s">
         <v>7</v>
       </c>
       <c r="F60" s="5" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
     </row>
     <row r="61" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A61" s="6" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C61" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D61" s="8" t="s">
+      <c r="D61" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="E61" s="9" t="s">
+      <c r="E61" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F61" s="5" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
     </row>
     <row r="62" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="B62" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="B62" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C62" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="D62" s="10" t="s">
-        <v>176</v>
-      </c>
-      <c r="E62" s="11" t="s">
+      <c r="C62" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="D62" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="E62" s="12" t="s">
         <v>7</v>
       </c>
       <c r="F62" s="5" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="63" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A63" s="15" t="s">
-        <v>178</v>
-      </c>
-      <c r="B63" s="21" t="s">
+      <c r="A63" s="16" t="s">
+        <v>182</v>
+      </c>
+      <c r="B63" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="C63" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="D63" s="18" t="s">
-        <v>179</v>
-      </c>
-      <c r="E63" s="17" t="s">
+      <c r="C63" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="D63" s="19" t="s">
+        <v>183</v>
+      </c>
+      <c r="E63" s="18" t="s">
         <v>7</v>
       </c>
       <c r="F63" s="5" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
     </row>
     <row r="64" spans="1:6" ht="87" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C64" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="E64" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F64" s="22" t="s">
-        <v>182</v>
+      <c r="F64" s="23" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="65" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A65" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="B65" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="B65" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="C65" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="D65" s="8" t="s">
-        <v>184</v>
-      </c>
-      <c r="E65" s="9" t="s">
+      <c r="C65" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="D65" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="E65" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F65" s="5" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
     </row>
     <row r="66" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="B66" s="12" t="s">
-        <v>149</v>
+        <v>190</v>
+      </c>
+      <c r="B66" s="13" t="s">
+        <v>152</v>
       </c>
       <c r="C66" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="E66" s="2" t="s">
         <v>7</v>
       </c>
       <c r="F66" s="5" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="6" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="B67" s="6" t="s">
         <v>42</v>
@@ -2607,39 +2628,39 @@
       <c r="C67" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D67" s="8" t="s">
-        <v>190</v>
-      </c>
-      <c r="E67" s="9" t="s">
+      <c r="D67" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="E67" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F67" s="5" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
     </row>
     <row r="68" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="B68" s="12" t="s">
+        <v>196</v>
+      </c>
+      <c r="B68" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D68" s="10" t="s">
-        <v>193</v>
-      </c>
-      <c r="E68" s="11" t="s">
+      <c r="D68" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="E68" s="12" t="s">
         <v>7</v>
       </c>
       <c r="F68" s="5" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
     </row>
     <row r="69" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A69" s="6" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B69" s="6" t="s">
         <v>21</v>
@@ -2647,42 +2668,42 @@
       <c r="C69" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D69" s="8" t="s">
+      <c r="D69" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="E69" s="9" t="s">
+      <c r="E69" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F69" s="5" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="B70" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="B70" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="C70" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="D70" s="8" t="s">
-        <v>197</v>
-      </c>
-      <c r="E70" s="9" t="s">
+      <c r="C70" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="D70" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="E70" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F70" s="5" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
     <row r="71" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A71" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="B71" s="12" t="s">
-        <v>164</v>
+        <v>203</v>
+      </c>
+      <c r="B71" s="13" t="s">
+        <v>168</v>
       </c>
       <c r="C71" s="6" t="s">
         <v>6</v>
@@ -2690,16 +2711,16 @@
       <c r="D71" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E71" s="13" t="s">
+      <c r="E71" s="14" t="s">
         <v>7</v>
       </c>
       <c r="F71" s="5" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
     </row>
     <row r="72" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="B72" s="1" t="s">
         <v>23</v>
@@ -2714,38 +2735,38 @@
         <v>7</v>
       </c>
       <c r="F72" s="5" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
     </row>
     <row r="73" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A73" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B73" s="12" t="s">
-        <v>149</v>
+      <c r="B73" s="13" t="s">
+        <v>152</v>
       </c>
       <c r="C73" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>203</v>
-      </c>
-      <c r="E73" s="13" t="s">
+        <v>207</v>
+      </c>
+      <c r="E73" s="14" t="s">
         <v>7</v>
       </c>
       <c r="F73" s="5" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="B74" s="12" t="s">
+        <v>209</v>
+      </c>
+      <c r="B74" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="C74" s="12" t="s">
-        <v>161</v>
+      <c r="C74" s="13" t="s">
+        <v>165</v>
       </c>
       <c r="D74" s="3">
         <v>230</v>
@@ -2754,58 +2775,58 @@
         <v>7</v>
       </c>
       <c r="F74" s="5" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" s="3" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="D75" s="25" t="s">
-        <v>222</v>
+        <v>165</v>
+      </c>
+      <c r="D75" s="26" t="s">
+        <v>226</v>
       </c>
       <c r="E75" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F75" s="5" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" s="3" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="D76" s="25" t="s">
-        <v>223</v>
+        <v>215</v>
+      </c>
+      <c r="D76" s="26" t="s">
+        <v>227</v>
       </c>
       <c r="E76" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F76" s="5" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" s="3" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="B77" s="3" t="s">
         <v>23</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="D77" s="3" t="s">
         <v>8</v>
@@ -2814,48 +2835,89 @@
         <v>7</v>
       </c>
       <c r="F77" s="5" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
     </row>
     <row r="78" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A78" s="3" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="B78" s="3" t="s">
         <v>31</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="D78" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="E78" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F78" s="23" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A79" s="24" t="s">
         <v>221</v>
       </c>
-      <c r="E78" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F78" s="22" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A79" s="23" t="s">
-        <v>217</v>
-      </c>
-      <c r="B79" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="C79" s="23" t="s">
+      <c r="B79" s="20" t="s">
+        <v>149</v>
+      </c>
+      <c r="C79" s="24" t="s">
         <v>6</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="E79" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F79" s="22" t="s">
-        <v>218</v>
-      </c>
+      <c r="F79" s="23" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A80" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C80" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D80" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="E80" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F80" s="5" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A81" s="16" t="s">
+        <v>133</v>
+      </c>
+      <c r="B81" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="C81" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="D81" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="E81" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="F81" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="G81" s="3"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -2989,6 +3051,9 @@
     <hyperlink ref="F79" r:id="rId128" display="https://www.openssl.org/" xr:uid="{59B58966-E35F-443B-9322-F153256A73B4}"/>
     <hyperlink ref="F2" r:id="rId129" xr:uid="{BD7ABBAE-8EE6-4349-90E3-6657A6659179}"/>
     <hyperlink ref="F4" r:id="rId130" display="https://www.bluez.org/" xr:uid="{D3C78CEA-BD7C-47D7-A10B-F7B3A0BCC41E}"/>
+    <hyperlink ref="F80" r:id="rId131" xr:uid="{39EC3A33-9F98-45A0-B03D-F21AD14EE922}"/>
+    <hyperlink ref="D81" r:id="rId132" display="https://github.com/rdkcentral/entservices-xcast/releases/tag/2.0.2" xr:uid="{D3A3079D-FC14-4915-8EED-F0B1DF4C5DC5}"/>
+    <hyperlink ref="F81" r:id="rId133" xr:uid="{AECE24CA-CDB4-4EA3-AC8A-CE94C83E9CB1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>